<commit_message>
Centroid file processing to add decoupling caps
</commit_message>
<xml_diff>
--- a/V14.0/Bill Of Materials APU - Routed.csv.xlsx
+++ b/V14.0/Bill Of Materials APU - Routed.csv.xlsx
@@ -388,7 +388,7 @@
     <t>Capacitors</t>
   </si>
   <si>
-    <t>One 100nF (0.1uF) capacitor for DIP ICs marked with extra DC near pin 1</t>
+    <t>DC-1,DC-2,DC-3,DC-4,DC-5</t>
   </si>
   <si>
     <t>K104K15X7RF53H5</t>
@@ -397,7 +397,7 @@
     <t>https://www.mouser.sg/ProductDetail/Vishay-BC-Components/K104K15X7RF53H5?qs=sYfpZ29HcUSlgH5bSUHkYw%3D%3D</t>
   </si>
   <si>
-    <t>Decoupling capacitors for each DC component</t>
+    <t>Decoupling capacitors for each DC component. One 100nF (0.1uF) capacitor for DIP ICs marked with extra DC near pin 1</t>
   </si>
   <si>
     <t>All with suffix CAP20</t>
@@ -406,7 +406,7 @@
     <t>149</t>
   </si>
   <si>
-    <t>One 100nF (0.1uF) capacitor for SMT ICs marked with extra SDC near pin 1</t>
+    <t>SDC-1,SDC-2,SDC-3,SDC-4,SDC-5,SDC-6,SDC-7,SDC-8,SDC-9,SDC-10,SDC-11,SDC-12,SDC-13,SDC-14,SDC-15,SDC-16,SDC-17,SDC-18,SDC-19,SDC-20,SDC-21,SDC-22,SDC-23,SDC-24,SDC-25,SDC-26,SDC-27,SDC-28,SDC-29,SDC-30,SDC-31,SDC-32,SDC-33,SDC-34,SDC-35,SDC-36,SDC-37,SDC-38,SDC-39,SDC-40,SDC-41,SDC-42,SDC-43,SDC-44,SDC-45,SDC-46,SDC-47,SDC-48,SDC-49,SDC-50,SDC-51,SDC-52,SDC-53,SDC-54,SDC-55,SDC-56,SDC-57,SDC-58,SDC-59,SDC-60,SDC-61,SDC-62,SDC-63,SDC-64,SDC-65,SDC-66,SDC-67,SDC-68,SDC-69,SDC-70,SDC-71,SDC-72,SDC-73,SDC-74,SDC-75,SDC-76,SDC-77,SDC-78,SDC-79,SDC-80,SDC-81,SDC-82,SDC-83,SDC-84,SDC-85,SDC-86,SDC-87,SDC-88,SDC-89,SDC-90,SDC-91,SDC-92,SDC-93,SDC-94,SDC-95,SDC-96,SDC-97,SDC-98,SDC-99,SDC-100,SDC-101,SDC-102,SDC-103,SDC-104,SDC-105,SDC-106,SDC-107,SDC-108,SDC-109,SDC-110,SDC-111,SDC-112,SDC-113,SDC-114,SDC-115,SDC-116,SDC-117,SDC-118,SDC-119,SDC-120,SDC-121,SDC-122,SDC-123,SDC-124,SDC-125,SDC-126,SDC-127,SDC-128,SDC-129,SDC-130,SDC-131,SDC-132,SDC-133,SDC-134,SDC-135,SDC-136,SDC-137,SDC-138,SDC-139,SDC-140,SDC-141,SDC-142,SDC-143,SDC-144,SDC-145,SDC-146,SDC-147,SDC-148,SDC-149</t>
   </si>
   <si>
     <t>CL05B104KO5NNNC</t>
@@ -415,7 +415,7 @@
     <t>https://www.mouser.sg/ProductDetail/Samsung-Electro-Mechanics/CL05B104KO5NNNC?qs=hqM3L16%252BxlfT2SKOuAUq6Q%3D%3D</t>
   </si>
   <si>
-    <t>Decoupling capacitors for each SDC component</t>
+    <t>Decoupling capacitors for each SDC component. One 100nF (0.1uF) capacitor for SMT ICs marked with extra SDC near pin 1</t>
   </si>
   <si>
     <t>All with suffix -CAP</t>
@@ -768,10 +768,10 @@
   <cols>
     <col min="1" max="1" width="17.28515625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="8.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="107.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="255.7109375" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="18.140625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="126.5703125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="90.5703125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="107.28515625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="25.85546875" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="11.140625" bestFit="1" customWidth="1"/>
   </cols>

</xml_diff>